<commit_message>
Update 26MMS0143-CISCO-Roster_Splunk Intermediate_15th to 17th June_VILT30007.xlsx
</commit_message>
<xml_diff>
--- a/26MMS0143-CISCO-Roster_Splunk Intermediate_15th to 17th June_VILT30007.xlsx
+++ b/26MMS0143-CISCO-Roster_Splunk Intermediate_15th to 17th June_VILT30007.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rpsconsulting-my.sharepoint.com/personal/arunkumar_h_rpsconsulting_in/Documents/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\VK_GIT\SPLK_CISCO_UK_15_06_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="8_{4F284087-A868-4CDF-A860-D34B152AC353}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E427CA21-E5B9-428C-8257-B76E4467D0C6}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80433B67-8609-4CBB-A1CD-AC8286615FDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{4ADD4C4D-4078-434B-99BB-934ACE1E975D}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{4ADD4C4D-4078-434B-99BB-934ACE1E975D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="lAB cREDENTIALS" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,8 +28,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -39,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="65">
   <si>
     <t>Start Date</t>
   </si>
@@ -141,13 +140,106 @@
   </si>
   <si>
     <t>Vivek Kumar Arora</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>Cloud Lab URL as follows: https://cloud4.rpsconsulting.in/console/</t>
+  </si>
+  <si>
+    <t>26MMS0143_U01</t>
+  </si>
+  <si>
+    <t>26MMS0143_U02</t>
+  </si>
+  <si>
+    <t>26MMS0143_U03</t>
+  </si>
+  <si>
+    <t>26MMS0143_U04</t>
+  </si>
+  <si>
+    <t>26MMS0143_U05</t>
+  </si>
+  <si>
+    <t>26MMS0143_U06</t>
+  </si>
+  <si>
+    <t>26MMS0143_U07</t>
+  </si>
+  <si>
+    <t>26MMS0143_U08</t>
+  </si>
+  <si>
+    <t>26MMS0143_U09</t>
+  </si>
+  <si>
+    <t>26MMS0143_U10</t>
+  </si>
+  <si>
+    <t>26MMS0143_U11</t>
+  </si>
+  <si>
+    <t>26MMS0143_U12</t>
+  </si>
+  <si>
+    <t>Username</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>Rps@Support9</t>
+  </si>
+  <si>
+    <t>Rps@Support10</t>
+  </si>
+  <si>
+    <t>Rps@Support11</t>
+  </si>
+  <si>
+    <t>Rps@Support12</t>
+  </si>
+  <si>
+    <t>Rps@Support13</t>
+  </si>
+  <si>
+    <t>Rps@Support14</t>
+  </si>
+  <si>
+    <t>Rps@Support15</t>
+  </si>
+  <si>
+    <t>Rps@Support16</t>
+  </si>
+  <si>
+    <t>Rps@Support17</t>
+  </si>
+  <si>
+    <t>Rps@Support18</t>
+  </si>
+  <si>
+    <t>Rps@Support19</t>
+  </si>
+  <si>
+    <t>Rps@Support20</t>
+  </si>
+  <si>
+    <t>Splunk credentials</t>
+  </si>
+  <si>
+    <t>Username: rps</t>
+  </si>
+  <si>
+    <t>Password: Rps@Support9</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -211,8 +303,35 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="13"/>
+      <color rgb="FF156082"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color rgb="FF156082"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -231,8 +350,20 @@
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="20">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -483,12 +614,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -514,12 +660,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -547,7 +687,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -589,6 +729,42 @@
     </xf>
     <xf numFmtId="15" fontId="4" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -926,31 +1102,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEE3727F-CED8-4986-B277-3B097141A157}">
   <dimension ref="A1:E23"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="38.6328125" customWidth="1"/>
-    <col min="2" max="2" width="22.453125" customWidth="1"/>
-    <col min="3" max="3" width="16.6328125" customWidth="1"/>
-    <col min="4" max="5" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="38.6640625" customWidth="1"/>
+    <col min="2" max="2" width="22.44140625" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" customWidth="1"/>
+    <col min="4" max="5" width="9.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-    </row>
-    <row r="2" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+    </row>
+    <row r="2" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
     </row>
-    <row r="3" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2"/>
       <c r="B3" s="3" t="s">
         <v>0</v>
@@ -961,9 +1137,9 @@
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
     </row>
-    <row r="4" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2"/>
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="32" t="s">
         <v>1</v>
       </c>
       <c r="C4" s="6">
@@ -972,29 +1148,29 @@
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
     </row>
-    <row r="5" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2"/>
-      <c r="B5" s="37" t="s">
+      <c r="B5" s="35" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="37" t="s">
+      <c r="C5" s="35" t="s">
         <v>33</v>
       </c>
       <c r="D5" s="5"/>
       <c r="E5" s="7"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
-      <c r="B6" s="35" t="s">
+      <c r="B6" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="36">
+      <c r="C6" s="34">
         <v>12</v>
       </c>
       <c r="D6" s="10"/>
       <c r="E6" s="10"/>
     </row>
-    <row r="7" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="8" t="s">
         <v>3</v>
@@ -1005,175 +1181,199 @@
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
       <c r="B8" s="1"/>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
       <c r="B9" s="1"/>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
     </row>
-    <row r="10" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2"/>
       <c r="B10" s="1"/>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
     </row>
-    <row r="11" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="13" t="s">
+    <row r="11" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="38">
+      <c r="C11" s="36">
         <v>46188</v>
       </c>
-      <c r="D11" s="39">
+      <c r="D11" s="37">
         <v>46189</v>
       </c>
-      <c r="E11" s="40">
+      <c r="E11" s="38">
         <v>46190</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="17" t="s">
+    <row r="12" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="15" t="s">
+      <c r="B12" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C12" s="24"/>
-      <c r="D12" s="25"/>
-      <c r="E12" s="26"/>
-    </row>
-    <row r="13" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="18" t="s">
+      <c r="C12" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="D12" s="23"/>
+      <c r="E12" s="24"/>
+    </row>
+    <row r="13" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="20"/>
-      <c r="D13" s="21"/>
-      <c r="E13" s="22"/>
-    </row>
-    <row r="14" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="23" t="s">
+      <c r="C13" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" s="19"/>
+      <c r="E13" s="20"/>
+    </row>
+    <row r="14" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="16" t="s">
+      <c r="B14" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="24"/>
-      <c r="D14" s="25"/>
-      <c r="E14" s="26"/>
-    </row>
-    <row r="15" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="27" t="s">
+      <c r="C14" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="D14" s="23"/>
+      <c r="E14" s="24"/>
+    </row>
+    <row r="15" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="C15" s="20"/>
-      <c r="D15" s="21"/>
-      <c r="E15" s="22"/>
-    </row>
-    <row r="16" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="28" t="s">
+      <c r="C15" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" s="19"/>
+      <c r="E15" s="20"/>
+    </row>
+    <row r="16" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="B16" s="29" t="s">
+      <c r="B16" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="C16" s="24"/>
-      <c r="D16" s="25"/>
-      <c r="E16" s="26"/>
-    </row>
-    <row r="17" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="30" t="s">
+      <c r="C16" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16" s="23"/>
+      <c r="E16" s="24"/>
+    </row>
+    <row r="17" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="B17" s="31" t="s">
+      <c r="B17" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="C17" s="20"/>
-      <c r="D17" s="21"/>
-      <c r="E17" s="22"/>
-    </row>
-    <row r="18" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="23" t="s">
+      <c r="C17" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="D17" s="19"/>
+      <c r="E17" s="20"/>
+    </row>
+    <row r="18" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="B18" s="16" t="s">
+      <c r="B18" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="24"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="26"/>
-    </row>
-    <row r="19" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="27" t="s">
+      <c r="C18" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="D18" s="23"/>
+      <c r="E18" s="24"/>
+    </row>
+    <row r="19" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="B19" s="19" t="s">
+      <c r="B19" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="C19" s="20"/>
-      <c r="D19" s="21"/>
-      <c r="E19" s="22"/>
-    </row>
-    <row r="20" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="32" t="s">
+      <c r="C19" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="D19" s="19"/>
+      <c r="E19" s="20"/>
+    </row>
+    <row r="20" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="16" t="s">
+      <c r="B20" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="C20" s="24"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="26"/>
-    </row>
-    <row r="21" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A21" s="18" t="s">
+      <c r="C20" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="D20" s="23"/>
+      <c r="E20" s="24"/>
+    </row>
+    <row r="21" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="19" t="s">
+      <c r="B21" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="C21" s="20"/>
-      <c r="D21" s="21"/>
-      <c r="E21" s="22"/>
-    </row>
-    <row r="22" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A22" s="23" t="s">
+      <c r="C21" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="D21" s="19"/>
+      <c r="E21" s="20"/>
+    </row>
+    <row r="22" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="B22" s="16" t="s">
+      <c r="B22" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="C22" s="24"/>
-      <c r="D22" s="25"/>
-      <c r="E22" s="26"/>
-    </row>
-    <row r="23" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A23" s="33" t="s">
+      <c r="C22" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="D22" s="23"/>
+      <c r="E22" s="24"/>
+    </row>
+    <row r="23" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="B23" s="19" t="s">
+      <c r="B23" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="C23" s="20"/>
-      <c r="D23" s="21"/>
-      <c r="E23" s="22"/>
+      <c r="C23" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="D23" s="19"/>
+      <c r="E23" s="20"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A12:B23">
@@ -1203,6 +1403,239 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{385AE8DE-0E61-4600-B23E-A498BB8A2986}">
+  <dimension ref="B3:E25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B6" s="41" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="41" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="50" t="s">
+        <v>48</v>
+      </c>
+      <c r="E6" s="50" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="B7" s="42" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="44" t="s">
+        <v>36</v>
+      </c>
+      <c r="E7" s="44" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="B8" s="45" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="E8" s="44" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="B9" s="47" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="46" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="44" t="s">
+        <v>38</v>
+      </c>
+      <c r="E9" s="44" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="B10" s="48" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" s="46" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="44" t="s">
+        <v>39</v>
+      </c>
+      <c r="E10" s="44" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B11" s="48" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="49" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="44" t="s">
+        <v>40</v>
+      </c>
+      <c r="E11" s="44" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="B12" s="42" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" s="43" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="E12" s="44" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="B13" s="47" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="46" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="44" t="s">
+        <v>42</v>
+      </c>
+      <c r="E13" s="44" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="B14" s="48" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="44" t="s">
+        <v>43</v>
+      </c>
+      <c r="E14" s="44" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="B15" s="45" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="46" t="s">
+        <v>29</v>
+      </c>
+      <c r="D15" s="44" t="s">
+        <v>44</v>
+      </c>
+      <c r="E15" s="44" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="B16" s="45" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="46" t="s">
+        <v>31</v>
+      </c>
+      <c r="D16" s="44" t="s">
+        <v>45</v>
+      </c>
+      <c r="E16" s="44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="B17" s="47" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" s="44" t="s">
+        <v>46</v>
+      </c>
+      <c r="E17" s="44" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="B18" s="47" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" s="46" t="s">
+        <v>30</v>
+      </c>
+      <c r="D18" s="44" t="s">
+        <v>47</v>
+      </c>
+      <c r="E18" s="44" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" ht="34.799999999999997" x14ac:dyDescent="0.3">
+      <c r="C23" s="51" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="C24" s="52" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" ht="34.799999999999997" x14ac:dyDescent="0.3">
+      <c r="C25" s="52" t="s">
+        <v>64</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="10" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="C18" r:id="rId1" xr:uid="{F3511E52-9532-4B81-9AF2-E3CA5289F6FA}"/>
+    <hyperlink ref="C9" r:id="rId2" xr:uid="{BFC17251-1EBB-4B89-95DE-371390C2169B}"/>
+    <hyperlink ref="C13" r:id="rId3" xr:uid="{5D955B97-1583-49EA-BF4D-EE69899A89DC}"/>
+    <hyperlink ref="C10" r:id="rId4" xr:uid="{50FFE1B8-152D-49DE-8849-C0B4220FC85C}"/>
+    <hyperlink ref="C11" r:id="rId5" xr:uid="{DB48A3FD-8C4E-4CB9-8FC9-C3FA3650977F}"/>
+    <hyperlink ref="C12" r:id="rId6" xr:uid="{C7FC3203-B172-437F-A7BC-EFD4919972E6}"/>
+    <hyperlink ref="C7" r:id="rId7" xr:uid="{0C89265C-44E7-478D-98C4-DC860435477C}"/>
+    <hyperlink ref="C8" r:id="rId8" xr:uid="{A356BC11-3371-4DA8-998B-432CFB198A58}"/>
+    <hyperlink ref="C14" r:id="rId9" xr:uid="{9BD40543-8029-4731-8DAE-D457BBC52F8D}"/>
+    <hyperlink ref="C17" r:id="rId10" xr:uid="{7DEB725A-2A55-489F-860A-212F24EEA44D}"/>
+    <hyperlink ref="C15" r:id="rId11" xr:uid="{359DC13D-8A68-410C-914D-1720ADE6E3A4}"/>
+    <hyperlink ref="C16" r:id="rId12" xr:uid="{BEFF5FF2-5BB7-4BF3-A412-68B005C0D73A}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{c8f49a32-fde3-48a5-9266-b5b0972a22dc}" enabled="1" method="Standard" siteId="{5ae1af62-9505-4097-a69a-c1553ef7840e}" contentBits="2" removed="0"/>

</xml_diff>